<commit_message>
ajustes de los nuevos valores, norm y idx
</commit_message>
<xml_diff>
--- a/results/logs/episode_metadata.xlsx
+++ b/results/logs/episode_metadata.xlsx
@@ -464,10 +464,10 @@
         <v>6981</v>
       </c>
       <c r="C2" t="n">
-        <v>7029</v>
+        <v>7005</v>
       </c>
       <c r="D2" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="E2" t="n">
         <v>0.6348337060527302</v>
@@ -514,7 +514,7 @@
         <v>6981</v>
       </c>
       <c r="B2" t="n">
-        <v>7029</v>
+        <v>7005</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
pruebas de trabajo relacionado para analisis cuantitaivio pero aun falta revisar detalles
</commit_message>
<xml_diff>
--- a/results/logs/episode_metadata.xlsx
+++ b/results/logs/episode_metadata.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E251"/>
+  <dimension ref="A1:E151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3003,1706 +3003,6 @@
         <v>239</v>
       </c>
       <c r="E151" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="n">
-        <v>150</v>
-      </c>
-      <c r="B152" t="n">
-        <v>0</v>
-      </c>
-      <c r="C152" t="n">
-        <v>239</v>
-      </c>
-      <c r="D152" t="n">
-        <v>239</v>
-      </c>
-      <c r="E152" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="n">
-        <v>151</v>
-      </c>
-      <c r="B153" t="n">
-        <v>0</v>
-      </c>
-      <c r="C153" t="n">
-        <v>239</v>
-      </c>
-      <c r="D153" t="n">
-        <v>239</v>
-      </c>
-      <c r="E153" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="n">
-        <v>152</v>
-      </c>
-      <c r="B154" t="n">
-        <v>0</v>
-      </c>
-      <c r="C154" t="n">
-        <v>239</v>
-      </c>
-      <c r="D154" t="n">
-        <v>239</v>
-      </c>
-      <c r="E154" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="n">
-        <v>153</v>
-      </c>
-      <c r="B155" t="n">
-        <v>0</v>
-      </c>
-      <c r="C155" t="n">
-        <v>239</v>
-      </c>
-      <c r="D155" t="n">
-        <v>239</v>
-      </c>
-      <c r="E155" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="n">
-        <v>154</v>
-      </c>
-      <c r="B156" t="n">
-        <v>0</v>
-      </c>
-      <c r="C156" t="n">
-        <v>239</v>
-      </c>
-      <c r="D156" t="n">
-        <v>239</v>
-      </c>
-      <c r="E156" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="n">
-        <v>155</v>
-      </c>
-      <c r="B157" t="n">
-        <v>0</v>
-      </c>
-      <c r="C157" t="n">
-        <v>239</v>
-      </c>
-      <c r="D157" t="n">
-        <v>239</v>
-      </c>
-      <c r="E157" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="n">
-        <v>156</v>
-      </c>
-      <c r="B158" t="n">
-        <v>0</v>
-      </c>
-      <c r="C158" t="n">
-        <v>239</v>
-      </c>
-      <c r="D158" t="n">
-        <v>239</v>
-      </c>
-      <c r="E158" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="n">
-        <v>157</v>
-      </c>
-      <c r="B159" t="n">
-        <v>0</v>
-      </c>
-      <c r="C159" t="n">
-        <v>239</v>
-      </c>
-      <c r="D159" t="n">
-        <v>239</v>
-      </c>
-      <c r="E159" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="n">
-        <v>158</v>
-      </c>
-      <c r="B160" t="n">
-        <v>0</v>
-      </c>
-      <c r="C160" t="n">
-        <v>239</v>
-      </c>
-      <c r="D160" t="n">
-        <v>239</v>
-      </c>
-      <c r="E160" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="n">
-        <v>159</v>
-      </c>
-      <c r="B161" t="n">
-        <v>0</v>
-      </c>
-      <c r="C161" t="n">
-        <v>239</v>
-      </c>
-      <c r="D161" t="n">
-        <v>239</v>
-      </c>
-      <c r="E161" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="n">
-        <v>160</v>
-      </c>
-      <c r="B162" t="n">
-        <v>0</v>
-      </c>
-      <c r="C162" t="n">
-        <v>239</v>
-      </c>
-      <c r="D162" t="n">
-        <v>239</v>
-      </c>
-      <c r="E162" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="n">
-        <v>161</v>
-      </c>
-      <c r="B163" t="n">
-        <v>0</v>
-      </c>
-      <c r="C163" t="n">
-        <v>239</v>
-      </c>
-      <c r="D163" t="n">
-        <v>239</v>
-      </c>
-      <c r="E163" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="n">
-        <v>162</v>
-      </c>
-      <c r="B164" t="n">
-        <v>0</v>
-      </c>
-      <c r="C164" t="n">
-        <v>239</v>
-      </c>
-      <c r="D164" t="n">
-        <v>239</v>
-      </c>
-      <c r="E164" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="n">
-        <v>163</v>
-      </c>
-      <c r="B165" t="n">
-        <v>0</v>
-      </c>
-      <c r="C165" t="n">
-        <v>239</v>
-      </c>
-      <c r="D165" t="n">
-        <v>239</v>
-      </c>
-      <c r="E165" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="n">
-        <v>164</v>
-      </c>
-      <c r="B166" t="n">
-        <v>0</v>
-      </c>
-      <c r="C166" t="n">
-        <v>239</v>
-      </c>
-      <c r="D166" t="n">
-        <v>239</v>
-      </c>
-      <c r="E166" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="n">
-        <v>165</v>
-      </c>
-      <c r="B167" t="n">
-        <v>0</v>
-      </c>
-      <c r="C167" t="n">
-        <v>239</v>
-      </c>
-      <c r="D167" t="n">
-        <v>239</v>
-      </c>
-      <c r="E167" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="n">
-        <v>166</v>
-      </c>
-      <c r="B168" t="n">
-        <v>0</v>
-      </c>
-      <c r="C168" t="n">
-        <v>239</v>
-      </c>
-      <c r="D168" t="n">
-        <v>239</v>
-      </c>
-      <c r="E168" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="n">
-        <v>167</v>
-      </c>
-      <c r="B169" t="n">
-        <v>0</v>
-      </c>
-      <c r="C169" t="n">
-        <v>239</v>
-      </c>
-      <c r="D169" t="n">
-        <v>239</v>
-      </c>
-      <c r="E169" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="n">
-        <v>168</v>
-      </c>
-      <c r="B170" t="n">
-        <v>0</v>
-      </c>
-      <c r="C170" t="n">
-        <v>239</v>
-      </c>
-      <c r="D170" t="n">
-        <v>239</v>
-      </c>
-      <c r="E170" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="n">
-        <v>169</v>
-      </c>
-      <c r="B171" t="n">
-        <v>0</v>
-      </c>
-      <c r="C171" t="n">
-        <v>239</v>
-      </c>
-      <c r="D171" t="n">
-        <v>239</v>
-      </c>
-      <c r="E171" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="n">
-        <v>170</v>
-      </c>
-      <c r="B172" t="n">
-        <v>0</v>
-      </c>
-      <c r="C172" t="n">
-        <v>239</v>
-      </c>
-      <c r="D172" t="n">
-        <v>239</v>
-      </c>
-      <c r="E172" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="n">
-        <v>171</v>
-      </c>
-      <c r="B173" t="n">
-        <v>0</v>
-      </c>
-      <c r="C173" t="n">
-        <v>239</v>
-      </c>
-      <c r="D173" t="n">
-        <v>239</v>
-      </c>
-      <c r="E173" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="n">
-        <v>172</v>
-      </c>
-      <c r="B174" t="n">
-        <v>0</v>
-      </c>
-      <c r="C174" t="n">
-        <v>239</v>
-      </c>
-      <c r="D174" t="n">
-        <v>239</v>
-      </c>
-      <c r="E174" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="n">
-        <v>173</v>
-      </c>
-      <c r="B175" t="n">
-        <v>0</v>
-      </c>
-      <c r="C175" t="n">
-        <v>239</v>
-      </c>
-      <c r="D175" t="n">
-        <v>239</v>
-      </c>
-      <c r="E175" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="n">
-        <v>174</v>
-      </c>
-      <c r="B176" t="n">
-        <v>0</v>
-      </c>
-      <c r="C176" t="n">
-        <v>239</v>
-      </c>
-      <c r="D176" t="n">
-        <v>239</v>
-      </c>
-      <c r="E176" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="n">
-        <v>175</v>
-      </c>
-      <c r="B177" t="n">
-        <v>0</v>
-      </c>
-      <c r="C177" t="n">
-        <v>239</v>
-      </c>
-      <c r="D177" t="n">
-        <v>239</v>
-      </c>
-      <c r="E177" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="n">
-        <v>176</v>
-      </c>
-      <c r="B178" t="n">
-        <v>0</v>
-      </c>
-      <c r="C178" t="n">
-        <v>239</v>
-      </c>
-      <c r="D178" t="n">
-        <v>239</v>
-      </c>
-      <c r="E178" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="n">
-        <v>177</v>
-      </c>
-      <c r="B179" t="n">
-        <v>0</v>
-      </c>
-      <c r="C179" t="n">
-        <v>239</v>
-      </c>
-      <c r="D179" t="n">
-        <v>239</v>
-      </c>
-      <c r="E179" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="n">
-        <v>178</v>
-      </c>
-      <c r="B180" t="n">
-        <v>0</v>
-      </c>
-      <c r="C180" t="n">
-        <v>239</v>
-      </c>
-      <c r="D180" t="n">
-        <v>239</v>
-      </c>
-      <c r="E180" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="n">
-        <v>179</v>
-      </c>
-      <c r="B181" t="n">
-        <v>0</v>
-      </c>
-      <c r="C181" t="n">
-        <v>239</v>
-      </c>
-      <c r="D181" t="n">
-        <v>239</v>
-      </c>
-      <c r="E181" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="n">
-        <v>180</v>
-      </c>
-      <c r="B182" t="n">
-        <v>0</v>
-      </c>
-      <c r="C182" t="n">
-        <v>239</v>
-      </c>
-      <c r="D182" t="n">
-        <v>239</v>
-      </c>
-      <c r="E182" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="n">
-        <v>181</v>
-      </c>
-      <c r="B183" t="n">
-        <v>0</v>
-      </c>
-      <c r="C183" t="n">
-        <v>239</v>
-      </c>
-      <c r="D183" t="n">
-        <v>239</v>
-      </c>
-      <c r="E183" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="n">
-        <v>182</v>
-      </c>
-      <c r="B184" t="n">
-        <v>0</v>
-      </c>
-      <c r="C184" t="n">
-        <v>239</v>
-      </c>
-      <c r="D184" t="n">
-        <v>239</v>
-      </c>
-      <c r="E184" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="n">
-        <v>183</v>
-      </c>
-      <c r="B185" t="n">
-        <v>0</v>
-      </c>
-      <c r="C185" t="n">
-        <v>239</v>
-      </c>
-      <c r="D185" t="n">
-        <v>239</v>
-      </c>
-      <c r="E185" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="n">
-        <v>184</v>
-      </c>
-      <c r="B186" t="n">
-        <v>0</v>
-      </c>
-      <c r="C186" t="n">
-        <v>239</v>
-      </c>
-      <c r="D186" t="n">
-        <v>239</v>
-      </c>
-      <c r="E186" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="n">
-        <v>185</v>
-      </c>
-      <c r="B187" t="n">
-        <v>0</v>
-      </c>
-      <c r="C187" t="n">
-        <v>239</v>
-      </c>
-      <c r="D187" t="n">
-        <v>239</v>
-      </c>
-      <c r="E187" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="n">
-        <v>186</v>
-      </c>
-      <c r="B188" t="n">
-        <v>0</v>
-      </c>
-      <c r="C188" t="n">
-        <v>239</v>
-      </c>
-      <c r="D188" t="n">
-        <v>239</v>
-      </c>
-      <c r="E188" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="n">
-        <v>187</v>
-      </c>
-      <c r="B189" t="n">
-        <v>0</v>
-      </c>
-      <c r="C189" t="n">
-        <v>239</v>
-      </c>
-      <c r="D189" t="n">
-        <v>239</v>
-      </c>
-      <c r="E189" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="n">
-        <v>188</v>
-      </c>
-      <c r="B190" t="n">
-        <v>0</v>
-      </c>
-      <c r="C190" t="n">
-        <v>239</v>
-      </c>
-      <c r="D190" t="n">
-        <v>239</v>
-      </c>
-      <c r="E190" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="n">
-        <v>189</v>
-      </c>
-      <c r="B191" t="n">
-        <v>0</v>
-      </c>
-      <c r="C191" t="n">
-        <v>239</v>
-      </c>
-      <c r="D191" t="n">
-        <v>239</v>
-      </c>
-      <c r="E191" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="n">
-        <v>190</v>
-      </c>
-      <c r="B192" t="n">
-        <v>0</v>
-      </c>
-      <c r="C192" t="n">
-        <v>239</v>
-      </c>
-      <c r="D192" t="n">
-        <v>239</v>
-      </c>
-      <c r="E192" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="n">
-        <v>191</v>
-      </c>
-      <c r="B193" t="n">
-        <v>0</v>
-      </c>
-      <c r="C193" t="n">
-        <v>239</v>
-      </c>
-      <c r="D193" t="n">
-        <v>239</v>
-      </c>
-      <c r="E193" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="n">
-        <v>192</v>
-      </c>
-      <c r="B194" t="n">
-        <v>0</v>
-      </c>
-      <c r="C194" t="n">
-        <v>239</v>
-      </c>
-      <c r="D194" t="n">
-        <v>239</v>
-      </c>
-      <c r="E194" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="n">
-        <v>193</v>
-      </c>
-      <c r="B195" t="n">
-        <v>0</v>
-      </c>
-      <c r="C195" t="n">
-        <v>239</v>
-      </c>
-      <c r="D195" t="n">
-        <v>239</v>
-      </c>
-      <c r="E195" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="n">
-        <v>194</v>
-      </c>
-      <c r="B196" t="n">
-        <v>0</v>
-      </c>
-      <c r="C196" t="n">
-        <v>239</v>
-      </c>
-      <c r="D196" t="n">
-        <v>239</v>
-      </c>
-      <c r="E196" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="n">
-        <v>195</v>
-      </c>
-      <c r="B197" t="n">
-        <v>0</v>
-      </c>
-      <c r="C197" t="n">
-        <v>239</v>
-      </c>
-      <c r="D197" t="n">
-        <v>239</v>
-      </c>
-      <c r="E197" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="n">
-        <v>196</v>
-      </c>
-      <c r="B198" t="n">
-        <v>0</v>
-      </c>
-      <c r="C198" t="n">
-        <v>239</v>
-      </c>
-      <c r="D198" t="n">
-        <v>239</v>
-      </c>
-      <c r="E198" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="n">
-        <v>197</v>
-      </c>
-      <c r="B199" t="n">
-        <v>0</v>
-      </c>
-      <c r="C199" t="n">
-        <v>239</v>
-      </c>
-      <c r="D199" t="n">
-        <v>239</v>
-      </c>
-      <c r="E199" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="n">
-        <v>198</v>
-      </c>
-      <c r="B200" t="n">
-        <v>0</v>
-      </c>
-      <c r="C200" t="n">
-        <v>239</v>
-      </c>
-      <c r="D200" t="n">
-        <v>239</v>
-      </c>
-      <c r="E200" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="n">
-        <v>199</v>
-      </c>
-      <c r="B201" t="n">
-        <v>0</v>
-      </c>
-      <c r="C201" t="n">
-        <v>239</v>
-      </c>
-      <c r="D201" t="n">
-        <v>239</v>
-      </c>
-      <c r="E201" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="n">
-        <v>200</v>
-      </c>
-      <c r="B202" t="n">
-        <v>0</v>
-      </c>
-      <c r="C202" t="n">
-        <v>239</v>
-      </c>
-      <c r="D202" t="n">
-        <v>239</v>
-      </c>
-      <c r="E202" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="n">
-        <v>201</v>
-      </c>
-      <c r="B203" t="n">
-        <v>0</v>
-      </c>
-      <c r="C203" t="n">
-        <v>239</v>
-      </c>
-      <c r="D203" t="n">
-        <v>239</v>
-      </c>
-      <c r="E203" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="n">
-        <v>202</v>
-      </c>
-      <c r="B204" t="n">
-        <v>0</v>
-      </c>
-      <c r="C204" t="n">
-        <v>239</v>
-      </c>
-      <c r="D204" t="n">
-        <v>239</v>
-      </c>
-      <c r="E204" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="n">
-        <v>203</v>
-      </c>
-      <c r="B205" t="n">
-        <v>0</v>
-      </c>
-      <c r="C205" t="n">
-        <v>239</v>
-      </c>
-      <c r="D205" t="n">
-        <v>239</v>
-      </c>
-      <c r="E205" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="n">
-        <v>204</v>
-      </c>
-      <c r="B206" t="n">
-        <v>0</v>
-      </c>
-      <c r="C206" t="n">
-        <v>239</v>
-      </c>
-      <c r="D206" t="n">
-        <v>239</v>
-      </c>
-      <c r="E206" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="n">
-        <v>205</v>
-      </c>
-      <c r="B207" t="n">
-        <v>0</v>
-      </c>
-      <c r="C207" t="n">
-        <v>239</v>
-      </c>
-      <c r="D207" t="n">
-        <v>239</v>
-      </c>
-      <c r="E207" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="n">
-        <v>206</v>
-      </c>
-      <c r="B208" t="n">
-        <v>0</v>
-      </c>
-      <c r="C208" t="n">
-        <v>239</v>
-      </c>
-      <c r="D208" t="n">
-        <v>239</v>
-      </c>
-      <c r="E208" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="n">
-        <v>207</v>
-      </c>
-      <c r="B209" t="n">
-        <v>0</v>
-      </c>
-      <c r="C209" t="n">
-        <v>239</v>
-      </c>
-      <c r="D209" t="n">
-        <v>239</v>
-      </c>
-      <c r="E209" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="n">
-        <v>208</v>
-      </c>
-      <c r="B210" t="n">
-        <v>0</v>
-      </c>
-      <c r="C210" t="n">
-        <v>239</v>
-      </c>
-      <c r="D210" t="n">
-        <v>239</v>
-      </c>
-      <c r="E210" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="n">
-        <v>209</v>
-      </c>
-      <c r="B211" t="n">
-        <v>0</v>
-      </c>
-      <c r="C211" t="n">
-        <v>239</v>
-      </c>
-      <c r="D211" t="n">
-        <v>239</v>
-      </c>
-      <c r="E211" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="n">
-        <v>210</v>
-      </c>
-      <c r="B212" t="n">
-        <v>0</v>
-      </c>
-      <c r="C212" t="n">
-        <v>239</v>
-      </c>
-      <c r="D212" t="n">
-        <v>239</v>
-      </c>
-      <c r="E212" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="n">
-        <v>211</v>
-      </c>
-      <c r="B213" t="n">
-        <v>0</v>
-      </c>
-      <c r="C213" t="n">
-        <v>239</v>
-      </c>
-      <c r="D213" t="n">
-        <v>239</v>
-      </c>
-      <c r="E213" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="n">
-        <v>212</v>
-      </c>
-      <c r="B214" t="n">
-        <v>0</v>
-      </c>
-      <c r="C214" t="n">
-        <v>239</v>
-      </c>
-      <c r="D214" t="n">
-        <v>239</v>
-      </c>
-      <c r="E214" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="n">
-        <v>213</v>
-      </c>
-      <c r="B215" t="n">
-        <v>0</v>
-      </c>
-      <c r="C215" t="n">
-        <v>239</v>
-      </c>
-      <c r="D215" t="n">
-        <v>239</v>
-      </c>
-      <c r="E215" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="n">
-        <v>214</v>
-      </c>
-      <c r="B216" t="n">
-        <v>0</v>
-      </c>
-      <c r="C216" t="n">
-        <v>239</v>
-      </c>
-      <c r="D216" t="n">
-        <v>239</v>
-      </c>
-      <c r="E216" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="n">
-        <v>215</v>
-      </c>
-      <c r="B217" t="n">
-        <v>0</v>
-      </c>
-      <c r="C217" t="n">
-        <v>239</v>
-      </c>
-      <c r="D217" t="n">
-        <v>239</v>
-      </c>
-      <c r="E217" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="n">
-        <v>216</v>
-      </c>
-      <c r="B218" t="n">
-        <v>0</v>
-      </c>
-      <c r="C218" t="n">
-        <v>239</v>
-      </c>
-      <c r="D218" t="n">
-        <v>239</v>
-      </c>
-      <c r="E218" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="n">
-        <v>217</v>
-      </c>
-      <c r="B219" t="n">
-        <v>0</v>
-      </c>
-      <c r="C219" t="n">
-        <v>239</v>
-      </c>
-      <c r="D219" t="n">
-        <v>239</v>
-      </c>
-      <c r="E219" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="n">
-        <v>218</v>
-      </c>
-      <c r="B220" t="n">
-        <v>0</v>
-      </c>
-      <c r="C220" t="n">
-        <v>239</v>
-      </c>
-      <c r="D220" t="n">
-        <v>239</v>
-      </c>
-      <c r="E220" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="n">
-        <v>219</v>
-      </c>
-      <c r="B221" t="n">
-        <v>0</v>
-      </c>
-      <c r="C221" t="n">
-        <v>239</v>
-      </c>
-      <c r="D221" t="n">
-        <v>239</v>
-      </c>
-      <c r="E221" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="n">
-        <v>220</v>
-      </c>
-      <c r="B222" t="n">
-        <v>0</v>
-      </c>
-      <c r="C222" t="n">
-        <v>239</v>
-      </c>
-      <c r="D222" t="n">
-        <v>239</v>
-      </c>
-      <c r="E222" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="n">
-        <v>221</v>
-      </c>
-      <c r="B223" t="n">
-        <v>0</v>
-      </c>
-      <c r="C223" t="n">
-        <v>239</v>
-      </c>
-      <c r="D223" t="n">
-        <v>239</v>
-      </c>
-      <c r="E223" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="n">
-        <v>222</v>
-      </c>
-      <c r="B224" t="n">
-        <v>0</v>
-      </c>
-      <c r="C224" t="n">
-        <v>239</v>
-      </c>
-      <c r="D224" t="n">
-        <v>239</v>
-      </c>
-      <c r="E224" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="n">
-        <v>223</v>
-      </c>
-      <c r="B225" t="n">
-        <v>0</v>
-      </c>
-      <c r="C225" t="n">
-        <v>239</v>
-      </c>
-      <c r="D225" t="n">
-        <v>239</v>
-      </c>
-      <c r="E225" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="n">
-        <v>224</v>
-      </c>
-      <c r="B226" t="n">
-        <v>0</v>
-      </c>
-      <c r="C226" t="n">
-        <v>239</v>
-      </c>
-      <c r="D226" t="n">
-        <v>239</v>
-      </c>
-      <c r="E226" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="n">
-        <v>225</v>
-      </c>
-      <c r="B227" t="n">
-        <v>0</v>
-      </c>
-      <c r="C227" t="n">
-        <v>239</v>
-      </c>
-      <c r="D227" t="n">
-        <v>239</v>
-      </c>
-      <c r="E227" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="n">
-        <v>226</v>
-      </c>
-      <c r="B228" t="n">
-        <v>0</v>
-      </c>
-      <c r="C228" t="n">
-        <v>239</v>
-      </c>
-      <c r="D228" t="n">
-        <v>239</v>
-      </c>
-      <c r="E228" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="n">
-        <v>227</v>
-      </c>
-      <c r="B229" t="n">
-        <v>0</v>
-      </c>
-      <c r="C229" t="n">
-        <v>239</v>
-      </c>
-      <c r="D229" t="n">
-        <v>239</v>
-      </c>
-      <c r="E229" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" t="n">
-        <v>228</v>
-      </c>
-      <c r="B230" t="n">
-        <v>0</v>
-      </c>
-      <c r="C230" t="n">
-        <v>239</v>
-      </c>
-      <c r="D230" t="n">
-        <v>239</v>
-      </c>
-      <c r="E230" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" t="n">
-        <v>229</v>
-      </c>
-      <c r="B231" t="n">
-        <v>0</v>
-      </c>
-      <c r="C231" t="n">
-        <v>239</v>
-      </c>
-      <c r="D231" t="n">
-        <v>239</v>
-      </c>
-      <c r="E231" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" t="n">
-        <v>230</v>
-      </c>
-      <c r="B232" t="n">
-        <v>0</v>
-      </c>
-      <c r="C232" t="n">
-        <v>239</v>
-      </c>
-      <c r="D232" t="n">
-        <v>239</v>
-      </c>
-      <c r="E232" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" t="n">
-        <v>231</v>
-      </c>
-      <c r="B233" t="n">
-        <v>0</v>
-      </c>
-      <c r="C233" t="n">
-        <v>239</v>
-      </c>
-      <c r="D233" t="n">
-        <v>239</v>
-      </c>
-      <c r="E233" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" t="n">
-        <v>232</v>
-      </c>
-      <c r="B234" t="n">
-        <v>0</v>
-      </c>
-      <c r="C234" t="n">
-        <v>239</v>
-      </c>
-      <c r="D234" t="n">
-        <v>239</v>
-      </c>
-      <c r="E234" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" t="n">
-        <v>233</v>
-      </c>
-      <c r="B235" t="n">
-        <v>0</v>
-      </c>
-      <c r="C235" t="n">
-        <v>239</v>
-      </c>
-      <c r="D235" t="n">
-        <v>239</v>
-      </c>
-      <c r="E235" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" t="n">
-        <v>234</v>
-      </c>
-      <c r="B236" t="n">
-        <v>0</v>
-      </c>
-      <c r="C236" t="n">
-        <v>239</v>
-      </c>
-      <c r="D236" t="n">
-        <v>239</v>
-      </c>
-      <c r="E236" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" t="n">
-        <v>235</v>
-      </c>
-      <c r="B237" t="n">
-        <v>0</v>
-      </c>
-      <c r="C237" t="n">
-        <v>239</v>
-      </c>
-      <c r="D237" t="n">
-        <v>239</v>
-      </c>
-      <c r="E237" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" t="n">
-        <v>236</v>
-      </c>
-      <c r="B238" t="n">
-        <v>0</v>
-      </c>
-      <c r="C238" t="n">
-        <v>239</v>
-      </c>
-      <c r="D238" t="n">
-        <v>239</v>
-      </c>
-      <c r="E238" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" t="n">
-        <v>237</v>
-      </c>
-      <c r="B239" t="n">
-        <v>0</v>
-      </c>
-      <c r="C239" t="n">
-        <v>239</v>
-      </c>
-      <c r="D239" t="n">
-        <v>239</v>
-      </c>
-      <c r="E239" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" t="n">
-        <v>238</v>
-      </c>
-      <c r="B240" t="n">
-        <v>0</v>
-      </c>
-      <c r="C240" t="n">
-        <v>239</v>
-      </c>
-      <c r="D240" t="n">
-        <v>239</v>
-      </c>
-      <c r="E240" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" t="n">
-        <v>239</v>
-      </c>
-      <c r="B241" t="n">
-        <v>0</v>
-      </c>
-      <c r="C241" t="n">
-        <v>239</v>
-      </c>
-      <c r="D241" t="n">
-        <v>239</v>
-      </c>
-      <c r="E241" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" t="n">
-        <v>240</v>
-      </c>
-      <c r="B242" t="n">
-        <v>0</v>
-      </c>
-      <c r="C242" t="n">
-        <v>239</v>
-      </c>
-      <c r="D242" t="n">
-        <v>239</v>
-      </c>
-      <c r="E242" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" t="n">
-        <v>241</v>
-      </c>
-      <c r="B243" t="n">
-        <v>0</v>
-      </c>
-      <c r="C243" t="n">
-        <v>239</v>
-      </c>
-      <c r="D243" t="n">
-        <v>239</v>
-      </c>
-      <c r="E243" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" t="n">
-        <v>242</v>
-      </c>
-      <c r="B244" t="n">
-        <v>0</v>
-      </c>
-      <c r="C244" t="n">
-        <v>239</v>
-      </c>
-      <c r="D244" t="n">
-        <v>239</v>
-      </c>
-      <c r="E244" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" t="n">
-        <v>243</v>
-      </c>
-      <c r="B245" t="n">
-        <v>0</v>
-      </c>
-      <c r="C245" t="n">
-        <v>239</v>
-      </c>
-      <c r="D245" t="n">
-        <v>239</v>
-      </c>
-      <c r="E245" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" t="n">
-        <v>244</v>
-      </c>
-      <c r="B246" t="n">
-        <v>0</v>
-      </c>
-      <c r="C246" t="n">
-        <v>239</v>
-      </c>
-      <c r="D246" t="n">
-        <v>239</v>
-      </c>
-      <c r="E246" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" t="n">
-        <v>245</v>
-      </c>
-      <c r="B247" t="n">
-        <v>0</v>
-      </c>
-      <c r="C247" t="n">
-        <v>239</v>
-      </c>
-      <c r="D247" t="n">
-        <v>239</v>
-      </c>
-      <c r="E247" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" t="n">
-        <v>246</v>
-      </c>
-      <c r="B248" t="n">
-        <v>0</v>
-      </c>
-      <c r="C248" t="n">
-        <v>239</v>
-      </c>
-      <c r="D248" t="n">
-        <v>239</v>
-      </c>
-      <c r="E248" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" t="n">
-        <v>247</v>
-      </c>
-      <c r="B249" t="n">
-        <v>0</v>
-      </c>
-      <c r="C249" t="n">
-        <v>239</v>
-      </c>
-      <c r="D249" t="n">
-        <v>239</v>
-      </c>
-      <c r="E249" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" t="n">
-        <v>248</v>
-      </c>
-      <c r="B250" t="n">
-        <v>0</v>
-      </c>
-      <c r="C250" t="n">
-        <v>239</v>
-      </c>
-      <c r="D250" t="n">
-        <v>239</v>
-      </c>
-      <c r="E250" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" t="n">
-        <v>249</v>
-      </c>
-      <c r="B251" t="n">
-        <v>0</v>
-      </c>
-      <c r="C251" t="n">
-        <v>239</v>
-      </c>
-      <c r="D251" t="n">
-        <v>239</v>
-      </c>
-      <c r="E251" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4750,11 +3050,11 @@
         <v>239</v>
       </c>
       <c r="C2" t="n">
-        <v>250</v>
+        <v>150</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 80, 81, 82, 83, 84, 85, 86, 87, 88, 89, 90, 91, 92, 93, 94, 95, 96, 97, 98, 99, 100, 101, 102, 103, 104, 105, 106, 107, 108, 109, 110, 111, 112, 113, 114, 115, 116, 117, 118, 119, 120, 121, 122, 123, 124, 125, 126, 127, 128, 129, 130, 131, 132, 133, 134, 135, 136, 137, 138, 139, 140, 141, 142, 143, 144, 145, 146, 147, 148, 149, 150, 151, 152, 153, 154, 155, 156, 157, 158, 159, 160, 161, 162, 163, 164, 165, 166, 167, 168, 169, 170, 171, 172, 173, 174, 175, 176, 177, 178, 179, 180, 181, 182, 183, 184, 185, 186, 187, 188, 189, 190, 191, 192, 193, 194, 195, 196, 197, 198, 199, 200, 201, 202, 203, 204, 205, 206, 207, 208, 209, 210, 211, 212, 213, 214, 215, 216, 217, 218, 219, 220, 221, 222, 223, 224, 225, 226, 227, 228, 229, 230, 231, 232, 233, 234, 235, 236, 237, 238, 239, 240, 241, 242, 243, 244, 245, 246, 247, 248, 249</t>
+          <t>0, 1, 2, 3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 30, 31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50, 51, 52, 53, 54, 55, 56, 57, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 80, 81, 82, 83, 84, 85, 86, 87, 88, 89, 90, 91, 92, 93, 94, 95, 96, 97, 98, 99, 100, 101, 102, 103, 104, 105, 106, 107, 108, 109, 110, 111, 112, 113, 114, 115, 116, 117, 118, 119, 120, 121, 122, 123, 124, 125, 126, 127, 128, 129, 130, 131, 132, 133, 134, 135, 136, 137, 138, 139, 140, 141, 142, 143, 144, 145, 146, 147, 148, 149</t>
         </is>
       </c>
     </row>
@@ -4767,12 +3067,12 @@
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Total Episodes: 250</t>
+          <t>Total Episodes: 150</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Unique Windows: 1, Max Freq: 250, Min Freq: 250, Avg Freq: 250.00</t>
+          <t>Unique Windows: 1, Max Freq: 150, Min Freq: 150, Avg Freq: 150.00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ajustes de balance de energia
</commit_message>
<xml_diff>
--- a/results/logs/episode_metadata.xlsx
+++ b/results/logs/episode_metadata.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,50 +461,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>235</v>
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>331</v>
+        <v>191</v>
       </c>
       <c r="D2" t="n">
-        <v>96</v>
+        <v>191</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7203244934421581</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="n">
-        <v>905</v>
-      </c>
-      <c r="C3" t="n">
-        <v>1001</v>
-      </c>
-      <c r="D3" t="n">
-        <v>96</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.3023325726318398</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="n">
-        <v>2895</v>
-      </c>
-      <c r="C4" t="n">
-        <v>2991</v>
-      </c>
-      <c r="D4" t="n">
-        <v>96</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.2360889769519761</v>
+        <v>0.8348421486656494</v>
       </c>
     </row>
   </sheetData>
@@ -518,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,10 +511,10 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>235</v>
+        <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>331</v>
+        <v>191</v>
       </c>
       <c r="C2" t="n">
         <v>1</v>
@@ -560,52 +526,20 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>905</v>
-      </c>
-      <c r="B3" t="n">
-        <v>1001</v>
-      </c>
-      <c r="C3" t="n">
-        <v>1</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SUMMARY</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Total Episodes: 1</t>
+        </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2895</v>
-      </c>
-      <c r="B4" t="n">
-        <v>2991</v>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>SUMMARY</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Total Episodes: 3</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Unique Windows: 3, Max Freq: 1, Min Freq: 1, Avg Freq: 1.00</t>
+          <t>Unique Windows: 1, Max Freq: 1, Min Freq: 1, Avg Freq: 1.00</t>
         </is>
       </c>
     </row>

</xml_diff>